<commit_message>
Translate all argument names, output columns and internal variables from Spanish to English (breaking change)
</commit_message>
<xml_diff>
--- a/inst/plantillas/plantilla_coshh.xlsx
+++ b/inst/plantillas/plantilla_coshh.xlsx
@@ -8,7 +8,7 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="COSHH_datos" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -550,14 +550,14 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>expoquimR · Plantilla COSHH Essentials</t>
+          <t>expoquimR · COSHH Essentials Template</t>
         </is>
       </c>
     </row>
     <row r="2" ht="50" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Instrucciones: una fila por sustancia. frases_h y frases_r: separadas por comas (ej. H315, H336). es_liquido: TRUE o FALSE. cantidad: Pequeña / Mediana / Grande. pulverulencia (solo sólidos): Baja / Media / Alta. t_ebullicion y t_proceso en °C (solo líquidos).</t>
+          <t>Instructions: one row per substance. h_phrases and r_phrases: comma-separated (e.g. H315, H336). is_liquid: TRUE or FALSE. quantity: Small / Medium / Large. dustiness (solids only): Low / Medium / High. boiling_point and process_temp in °C (liquids only).</t>
         </is>
       </c>
       <c r="B2" s="3" t="n"/>
@@ -571,49 +571,49 @@
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>sustancia</t>
+          <t>substance</t>
         </is>
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>frases_h</t>
+          <t>h_phrases</t>
         </is>
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>frases_r</t>
+          <t>r_phrases</t>
         </is>
       </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
-          <t>cantidad</t>
+          <t>quantity</t>
         </is>
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t>es_liquido</t>
+          <t>is_liquid</t>
         </is>
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
-          <t>t_ebullicion</t>
+          <t>boiling_point</t>
         </is>
       </c>
       <c r="G3" s="5" t="inlineStr">
         <is>
-          <t>t_proceso</t>
+          <t>process_temp</t>
         </is>
       </c>
       <c r="H3" s="5" t="inlineStr">
         <is>
-          <t>pulverulencia</t>
+          <t>dustiness</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>Tolueno</t>
+          <t>Toluene</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
@@ -624,7 +624,7 @@
       <c r="C4" s="6" t="inlineStr"/>
       <c r="D4" s="6" t="inlineStr">
         <is>
-          <t>Mediana</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E4" s="6" t="inlineStr">
@@ -643,7 +643,7 @@
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>Cemento</t>
+          <t>Cement</t>
         </is>
       </c>
       <c r="B5" s="6" t="inlineStr">
@@ -654,7 +654,7 @@
       <c r="C5" s="6" t="inlineStr"/>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>Grande</t>
+          <t>Large</t>
         </is>
       </c>
       <c r="E5" s="6" t="inlineStr">
@@ -666,14 +666,14 @@
       <c r="G5" s="6" t="inlineStr"/>
       <c r="H5" s="6" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>High</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>Acido sulfurico</t>
+          <t>Sulfuric acid</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr"/>
@@ -684,7 +684,7 @@
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>Pequeña</t>
+          <t>Small</t>
         </is>
       </c>
       <c r="E6" s="6" t="inlineStr">
@@ -696,7 +696,7 @@
       <c r="G6" s="6" t="inlineStr"/>
       <c r="H6" s="6" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -726,92 +726,92 @@
     <row r="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>Campo</t>
+          <t>Field</t>
         </is>
       </c>
       <c r="B1" s="7" t="inlineStr">
         <is>
-          <t>Valores aceptados</t>
+          <t>Accepted values</t>
         </is>
       </c>
       <c r="C1" s="7" t="inlineStr">
         <is>
-          <t>Obligatorio</t>
+          <t>Required</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>sustancia</t>
+          <t>substance</t>
         </is>
       </c>
       <c r="B2" s="8" t="inlineStr">
         <is>
-          <t>Texto libre</t>
+          <t>Free text</t>
         </is>
       </c>
       <c r="C2" s="8" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="8" t="inlineStr">
         <is>
-          <t>frases_h</t>
+          <t>h_phrases</t>
         </is>
       </c>
       <c r="B3" s="8" t="inlineStr">
         <is>
-          <t>Codigos H separados por comas</t>
+          <t>H codes separated by commas</t>
         </is>
       </c>
       <c r="C3" s="8" t="inlineStr">
         <is>
-          <t>No (si hay frases_r)</t>
+          <t>No (if r_phrases is provided)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
-          <t>frases_r</t>
+          <t>r_phrases</t>
         </is>
       </c>
       <c r="B4" s="8" t="inlineStr">
         <is>
-          <t>Codigos R separados por comas</t>
+          <t>R codes separated by commas</t>
         </is>
       </c>
       <c r="C4" s="8" t="inlineStr">
         <is>
-          <t>No (si hay frases_h)</t>
+          <t>No (if h_phrases is provided)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="8" t="inlineStr">
         <is>
-          <t>cantidad</t>
+          <t>quantity</t>
         </is>
       </c>
       <c r="B5" s="8" t="inlineStr">
         <is>
-          <t>Pequeña / Mediana / Grande</t>
+          <t>Small / Medium / Large</t>
         </is>
       </c>
       <c r="C5" s="8" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="8" t="inlineStr">
         <is>
-          <t>es_liquido</t>
+          <t>is_liquid</t>
         </is>
       </c>
       <c r="B6" s="8" t="inlineStr">
@@ -821,58 +821,58 @@
       </c>
       <c r="C6" s="8" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="8" t="inlineStr">
         <is>
-          <t>t_ebullicion</t>
+          <t>boiling_point</t>
         </is>
       </c>
       <c r="B7" s="8" t="inlineStr">
         <is>
-          <t>Numero en °C</t>
+          <t>Number in °C</t>
         </is>
       </c>
       <c r="C7" s="8" t="inlineStr">
         <is>
-          <t>Solo si es_liquido=TRUE</t>
+          <t>Only if is_liquid=TRUE</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="8" t="inlineStr">
         <is>
-          <t>t_proceso</t>
+          <t>process_temp</t>
         </is>
       </c>
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t>Numero en °C</t>
+          <t>Number in °C</t>
         </is>
       </c>
       <c r="C8" s="8" t="inlineStr">
         <is>
-          <t>Solo si es_liquido=TRUE</t>
+          <t>Only if is_liquid=TRUE</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>pulverulencia</t>
+          <t>dustiness</t>
         </is>
       </c>
       <c r="B9" s="8" t="inlineStr">
         <is>
-          <t>Baja / Media / Alta</t>
+          <t>Low / Medium / High</t>
         </is>
       </c>
       <c r="C9" s="8" t="inlineStr">
         <is>
-          <t>Solo si es_liquido=FALSE</t>
+          <t>Only if is_liquid=FALSE</t>
         </is>
       </c>
     </row>

</xml_diff>